<commit_message>
Corregir parse_euro_amount: eliminar str() innecesario
El str() convertia floats de Excel a strings, y el regex rompia
valores como 23917.620000000003 -> 23917620000000004.

Corregido en: extraer_datos.py, regenerar_dashboard.py,
crear_excel_completo.py

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/ECO_STRUCT_Datos.xlsx
+++ b/ECO_STRUCT_Datos.xlsx
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>2.391762e+16</v>
+        <v>23917.62</v>
       </c>
       <c r="D5" s="6">
         <f>C5/C24</f>
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>6.327734e+16</v>
+        <v>63277.34</v>
       </c>
       <c r="D9" s="6">
         <f>C9/C24</f>
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1.1643226e+16</v>
+        <v>116432.26</v>
       </c>
       <c r="D12" s="6">
         <f>C12/C24</f>
@@ -1728,7 +1728,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>8883470999999999</v>
+        <v>88834.70999999999</v>
       </c>
       <c r="D17" s="6">
         <f>C17/C24</f>

</xml_diff>